<commit_message>
Reject duplicate member ID when admin adds a member
</commit_message>
<xml_diff>
--- a/docs/Testing Document.xlsx
+++ b/docs/Testing Document.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.6328125" customWidth="1" min="1" max="1"/>
@@ -1368,6 +1368,116 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TC30</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Register New Member Account</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>1. On the login screen, click "New here? Create a member account"
+2. Fill in Username, Password, Full Name, Email, Date of Birth, Address
+3. Choose Membership Type
+4. Click "Create Account"</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Username: newuser01
+Password: pass123
+Full Name: New User
+Email: newuser01@ut.edu.vn
+Date of Birth: 2002-03-04
+Address: 1 Test St
+Membership Type: Standard</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Account is created (new Member ID shown), and the user is logged in immediately as a Member. Registering again with the same username shows an error instead of creating a duplicate account.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TC31</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Add Book (Duplicate Code)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as Admin
+2. Click "Book Management" -&gt; "Add book"
+3. Enter a Code that already exists
+4. Fill remaining fields
+5. Submit</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Code: BK001 (already exists)
+Title: Duplicate Test
+Author: Test
+Category: Test
+Publisher: Test
+Quantity: 1</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Popup/message shows "Book code 'BK001' already exists." and no duplicate book is added to the list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TC32</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Add Member (Duplicate Member ID)</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>1. Log in as Admin
+2. Click "Member Management" -&gt; "Add member"
+3. Enter a Member ID that already exists (but a new Username)
+4. Fill remaining fields
+5. Submit</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Member ID: LIB001 (already exists)
+Username: brandnewuser
+Password: 123456
+Full Name: Duplicate ID Test
+Email: dup@ut.edu.vn
+Date of Birth: 2000-01-01
+Address: Test
+Membership Type: Standard</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Popup/message shows "Member ID 'LIB001' already exists." and no duplicate member is added to the list.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>